<commit_message>
Updated duplicate reference fix, kill process
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\UiPath\AZ-Application Review Process_Dispatcher\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Az_Application-Review-Process_Dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD0592A-5225-43EB-8167-49FF2348D99F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F48EB40-A0D9-4E23-A702-0118BC0C2A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="55">
   <si>
     <t>Name</t>
   </si>
@@ -85,9 +85,6 @@
   </si>
   <si>
     <t>logF_BusinessProcessName</t>
-  </si>
-  <si>
-    <t>Framework</t>
   </si>
   <si>
     <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
@@ -159,9 +156,6 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>ProcessABCQueue</t>
-  </si>
-  <si>
     <t>ManagerName</t>
   </si>
   <si>
@@ -186,7 +180,16 @@
     <t>FailureEmailBody</t>
   </si>
   <si>
-    <t>Hello,&lt;br&gt;AZ-Application Review Process_Dispatcher failed to process. Reason:&lt;br&gt;&lt;Reason&gt;&lt;br&gt;&lt;br&gt;Thanks,Bot</t>
+    <t>The {0} process has encountered a System Error.\n\nMachine Name: {1} \n\nLAN ID: {2} \n\nException Timestamp: {3} \n\nTransaction Reference: {4} \n\nException Message: {5} \n\nException Source: {6}</t>
+  </si>
+  <si>
+    <t>AZ-Application Review Process_Dispatcher</t>
+  </si>
+  <si>
+    <t>AZ_ApplicationReview</t>
+  </si>
+  <si>
+    <t>InputFilesStorageBucketName</t>
   </si>
 </sst>
 </file>
@@ -607,22 +610,21 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="45">
       <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
@@ -631,10 +633,10 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1639,7 +1641,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z988"/>
+  <dimension ref="A1:Z987"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -1690,18 +1692,18 @@
         <v>0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1725,7 +1727,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -1747,7 +1749,7 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
@@ -1758,7 +1760,7 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
@@ -1769,70 +1771,70 @@
         <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="17" spans="1:3" ht="45">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B17" t="b">
         <v>0</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2802,7 +2804,6 @@
     <row r="985" ht="14.25" customHeight="1"/>
     <row r="986" ht="14.25" customHeight="1"/>
     <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2828,7 +2829,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
@@ -2858,53 +2859,60 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
+        <v>54</v>
+      </c>
+    </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Updated Config for email template for html format
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Az_Application-Review-Process_Dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F48EB40-A0D9-4E23-A702-0118BC0C2A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC3403E-8D96-4B6F-B1B1-EBC645C7F4C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -180,9 +180,6 @@
     <t>FailureEmailBody</t>
   </si>
   <si>
-    <t>The {0} process has encountered a System Error.\n\nMachine Name: {1} \n\nLAN ID: {2} \n\nException Timestamp: {3} \n\nTransaction Reference: {4} \n\nException Message: {5} \n\nException Source: {6}</t>
-  </si>
-  <si>
     <t>AZ-Application Review Process_Dispatcher</t>
   </si>
   <si>
@@ -190,6 +187,9 @@
   </si>
   <si>
     <t>InputFilesStorageBucketName</t>
+  </si>
+  <si>
+    <t>The {0} process has encountered a System Error.&lt;br&gt;&lt;br&gt;Machine Name: {1} &lt;br&gt;&lt;br&gt;LAN ID: {2} \n\nException Timestamp: {3} &lt;br&gt;&lt;br&gt;Transaction Reference: {4} &lt;br&gt;&lt;br&gt;Exception Message: {5} &lt;br&gt;&lt;br&gt;Exception Source: {6}</t>
   </si>
 </sst>
 </file>
@@ -613,7 +613,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
@@ -633,7 +633,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -1834,7 +1834,7 @@
         <v>50</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2907,10 +2907,10 @@
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Updated code to include last upload Date in Queue reference
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Az_Application-Review-Process_Dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC3403E-8D96-4B6F-B1B1-EBC645C7F4C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D2A4FA-30CD-487A-AC6E-D948C464C093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13950" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4260" yWindow="2310" windowWidth="20190" windowHeight="9720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="56">
   <si>
     <t>Name</t>
   </si>
@@ -190,6 +190,9 @@
   </si>
   <si>
     <t>The {0} process has encountered a System Error.&lt;br&gt;&lt;br&gt;Machine Name: {1} &lt;br&gt;&lt;br&gt;LAN ID: {2} \n\nException Timestamp: {3} &lt;br&gt;&lt;br&gt;Transaction Reference: {4} &lt;br&gt;&lt;br&gt;Exception Message: {5} &lt;br&gt;&lt;br&gt;Exception Source: {6}</t>
+  </si>
+  <si>
+    <t>PersonNameSelector</t>
   </si>
 </sst>
 </file>
@@ -2913,7 +2916,14 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+    </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
updates to Column numnber and rows in Dispatcher
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Az_Application-Review-Process_Dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D2A4FA-30CD-487A-AC6E-D948C464C093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B51AEA6A-FA3E-4564-A69E-60DA1C6C9944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4260" yWindow="2310" windowWidth="20190" windowHeight="9720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="60">
   <si>
     <t>Name</t>
   </si>
@@ -193,6 +193,18 @@
   </si>
   <si>
     <t>PersonNameSelector</t>
+  </si>
+  <si>
+    <t>Yardi_DetailsIndexNumber</t>
+  </si>
+  <si>
+    <t>Yardi_CaseLinkIndexNumber</t>
+  </si>
+  <si>
+    <t>Yardi_ColumnToRemove</t>
+  </si>
+  <si>
+    <t>Yardi_UnwantedRowsWithDashboardTitles</t>
   </si>
 </sst>
 </file>
@@ -2924,10 +2936,38 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" t="s">
+        <v>59</v>
+      </c>
+    </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>